<commit_message>
docs(sheet): sample sheet header tiếng Việt đầy đủ
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sheet-mau/sheet-mau.xlsx
+++ b/docs/sheet-mau/sheet-mau.xlsx
@@ -321,7 +321,7 @@
     </comment>
     <comment ref="E2" authorId="0" shapeId="0">
       <text>
-        <t>[chromaKeyAuto] 4 màu ứng viên (hex, cách nhau dấu phẩy). App tự chọn màu gần nhất cho TỪNG video.</t>
+        <t>[Kiểu render = chromaKeyAuto] 4 màu ứng viên (hex, cách nhau dấu phẩy). App tự chọn màu gần nhất cho TỪNG video.</t>
       </text>
     </comment>
     <comment ref="F2" authorId="0" shapeId="0">
@@ -351,12 +351,12 @@
     </comment>
     <comment ref="K2" authorId="0" shapeId="0">
       <text>
-        <t>[keepColor] Chiều cao dải giữ (px), khi keepCrop=true.</t>
+        <t>[keepColor] Chiều cao dải giữ (px), khi bật cắt.</t>
       </text>
     </comment>
     <comment ref="L2" authorId="0" shapeId="0">
       <text>
-        <t>[keepColor] Vị trí y bắt đầu cắt (px), khi keepCrop=true.</t>
+        <t>[keepColor] Vị trí y bắt đầu cắt (px), khi bật cắt.</t>
       </text>
     </comment>
     <comment ref="M2" authorId="0" shapeId="0">
@@ -754,87 +754,87 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>sheetName</t>
+          <t>Tên kênh</t>
         </is>
       </c>
       <c r="B2" s="8" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>Bật</t>
         </is>
       </c>
       <c r="C2" s="8" t="inlineStr">
         <is>
-          <t>videosPerDay</t>
+          <t>Video mỗi ngày</t>
         </is>
       </c>
       <c r="D2" s="8" t="inlineStr">
         <is>
-          <t>renderMode</t>
+          <t>Kiểu render</t>
         </is>
       </c>
       <c r="E2" s="9" t="inlineStr">
         <is>
-          <t>chromaPalette</t>
+          <t>Bảng màu tự dò</t>
         </is>
       </c>
       <c r="F2" s="10" t="inlineStr">
         <is>
-          <t>chromaColor</t>
+          <t>Màu phông</t>
         </is>
       </c>
       <c r="G2" s="10" t="inlineStr">
         <is>
-          <t>chromaSimilarity</t>
+          <t>Độ nhạy chroma</t>
         </is>
       </c>
       <c r="H2" s="11" t="inlineStr">
         <is>
-          <t>opacity</t>
+          <t>Độ mờ</t>
         </is>
       </c>
       <c r="I2" s="12" t="inlineStr">
         <is>
-          <t>keepColors</t>
+          <t>Màu giữ lại</t>
         </is>
       </c>
       <c r="J2" s="12" t="inlineStr">
         <is>
-          <t>keepCrop</t>
+          <t>Bật cắt (giữ màu)</t>
         </is>
       </c>
       <c r="K2" s="12" t="inlineStr">
         <is>
-          <t>keepHeight</t>
+          <t>Chiều cao cắt (giữ màu)</t>
         </is>
       </c>
       <c r="L2" s="12" t="inlineStr">
         <is>
-          <t>keepYOffset</t>
+          <t>Vị trí Y (giữ màu)</t>
         </is>
       </c>
       <c r="M2" s="12" t="inlineStr">
         <is>
-          <t>keepSimilarity</t>
+          <t>Độ nhạy giữ màu</t>
         </is>
       </c>
       <c r="N2" s="12" t="inlineStr">
         <is>
-          <t>keepAddDarkLayer</t>
+          <t>Lớp nền tối</t>
         </is>
       </c>
       <c r="O2" s="13" t="inlineStr">
         <is>
-          <t>cropHeight</t>
+          <t>Chiều cao cắt</t>
         </is>
       </c>
       <c r="P2" s="13" t="inlineStr">
         <is>
-          <t>cropYOffset</t>
+          <t>Vị trí Y cắt</t>
         </is>
       </c>
       <c r="Q2" s="14" t="inlineStr">
         <is>
-          <t>proxy</t>
+          <t>Proxy tải</t>
         </is>
       </c>
     </row>
@@ -1168,7 +1168,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Tab ⚙config: mỗi dòng = 1 kênh. Dòng 1 = nhóm theo mode (tô màu), dòng 2 = tên cột (app đọc, GIỮ tiếng Anh).</t>
+          <t>Tab ⚙config: mỗi dòng = 1 kênh. Dòng 1 = nhóm theo mode (tô màu), dòng 2 = tên cột (tiếng Việt). Rê chuột vào tiêu đề cột để xem chú thích.</t>
         </is>
       </c>
     </row>
@@ -1196,7 +1196,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>sheetName, enabled, videosPerDay, renderMode</t>
+          <t>Tên kênh, Bật, Video mỗi ngày, Kiểu render</t>
         </is>
       </c>
     </row>
@@ -1208,7 +1208,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>chromaPalette — 4 màu ứng viên; app tự dò màu gần nhất cho từng video</t>
+          <t>Bảng màu tự dò — 4 màu ứng viên; app tự dò màu gần nhất cho từng video</t>
         </is>
       </c>
     </row>
@@ -1220,7 +1220,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>chromaColor, chromaSimilarity — xóa 1 màu phông cố định</t>
+          <t>Màu phông, Độ nhạy chroma — xóa 1 màu phông cố định</t>
         </is>
       </c>
     </row>
@@ -1232,7 +1232,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>opacity — phủ overlay mờ lên nền</t>
+          <t>Độ mờ — phủ overlay mờ lên nền</t>
         </is>
       </c>
     </row>
@@ -1244,7 +1244,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>keepColors, keepCrop, keepHeight, keepYOffset, keepSimilarity, keepAddDarkLayer — chỉ giữ lại vài màu</t>
+          <t>Màu giữ lại, Bật cắt (giữ màu), Chiều cao/Vị trí Y (giữ màu), Độ nhạy giữ màu, Lớp nền tối</t>
         </is>
       </c>
     </row>
@@ -1256,7 +1256,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>cropHeight, cropYOffset — cắt một dải overlay</t>
+          <t>Chiều cao cắt, Vị trí Y cắt — cắt một dải overlay</t>
         </is>
       </c>
     </row>
@@ -1268,7 +1268,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>proxy — chỉ dùng khi TẢI video (yt-dlp)</t>
+          <t>Proxy tải — chỉ dùng khi TẢI video (yt-dlp)</t>
         </is>
       </c>
     </row>

</xml_diff>